<commit_message>
feat: implement frontend routing and core admin/teacher/student panel navigation structures
</commit_message>
<xml_diff>
--- a/ExamGuardAI_Question_Import_Template.xlsx
+++ b/ExamGuardAI_Question_Import_Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>question</t>
   </si>
@@ -32,6 +32,84 @@
   </si>
   <si>
     <t>correct_option</t>
+  </si>
+  <si>
+    <t>Which of the following data structures operates on a Last-In, First-Out (LIFO) basis?</t>
+  </si>
+  <si>
+    <t>What is the primary characteristic of a standard Queue data structure?</t>
+  </si>
+  <si>
+    <t>Which data structure is typically used to implement Breadth-First Search (BFS) on a graph?</t>
+  </si>
+  <si>
+    <t>What is the time complexity of pushing an element onto a stack implemented using an array (assuming no resizing is needed)?</t>
+  </si>
+  <si>
+    <t>Which of the following is a common application of a Stack data structure?</t>
+  </si>
+  <si>
+    <t>Queue</t>
+  </si>
+  <si>
+    <t>First-In, First-Out (FIFO)</t>
+  </si>
+  <si>
+    <t>Stack</t>
+  </si>
+  <si>
+    <t>O(N)</t>
+  </si>
+  <si>
+    <t>Job scheduling in operating systems</t>
+  </si>
+  <si>
+    <t>Last-In, First-Out (LIFO)</t>
+  </si>
+  <si>
+    <t>Heap</t>
+  </si>
+  <si>
+    <t>O(log N)</t>
+  </si>
+  <si>
+    <t>Balancing symbols / Parentheses matching</t>
+  </si>
+  <si>
+    <t>Array</t>
+  </si>
+  <si>
+    <t>Random access of elements</t>
+  </si>
+  <si>
+    <t>O(1)</t>
+  </si>
+  <si>
+    <t>Breadth-First Search traversal</t>
+  </si>
+  <si>
+    <t>Linked List</t>
+  </si>
+  <si>
+    <t>Sorted ordering of elements</t>
+  </si>
+  <si>
+    <t>Binary Search Tree</t>
+  </si>
+  <si>
+    <t>O(N log N)</t>
+  </si>
+  <si>
+    <t>Serving print requests in a print queue</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
@@ -363,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -386,6 +464,106 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>